<commit_message>
chore: update estacionesSAMADB.xlsx with latest data
</commit_message>
<xml_diff>
--- a/estacionesSAMADB.xlsx
+++ b/estacionesSAMADB.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmonto37\Documents\SAMA\Solicitud_Pronosticos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmonto37\Documents\SAMA\Movimientos Masa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EECE6453-899E-45EE-9D50-6EDA155F9F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F47007-04BC-4AE5-9D69-F8E8269B3DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Instrumentos_actualizado!$A$1:$L$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Instrumentos_actualizado!$A$1:$L$127</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -33,12 +33,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="431">
   <si>
     <t>GRUPO</t>
   </si>
@@ -1298,6 +1301,48 @@
   </si>
   <si>
     <t>Río Tamar - Vereda Tamar</t>
+  </si>
+  <si>
+    <t>Casco urbano - Gomez plata</t>
+  </si>
+  <si>
+    <t>sp_164</t>
+  </si>
+  <si>
+    <t>sp_165</t>
+  </si>
+  <si>
+    <t>sp_166</t>
+  </si>
+  <si>
+    <t>sp_167</t>
+  </si>
+  <si>
+    <t>sp_168</t>
+  </si>
+  <si>
+    <t>GOMEZ PLATA</t>
+  </si>
+  <si>
+    <t>Vegachí</t>
+  </si>
+  <si>
+    <t>VEGACHI</t>
+  </si>
+  <si>
+    <t>Fredonia</t>
+  </si>
+  <si>
+    <t>FREDONIA</t>
+  </si>
+  <si>
+    <t>Fredonia2</t>
+  </si>
+  <si>
+    <t>Pueblorrico</t>
+  </si>
+  <si>
+    <t>PLUEBLORRICO</t>
   </si>
 </sst>
 </file>
@@ -1467,12 +1512,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2283,7 +2329,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2589,50 +2635,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -2990,11 +3039,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ127"/>
+  <dimension ref="A1:AQ132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="48.75" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.26953125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.54296875" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.26953125" style="3" customWidth="1"/>
     <col min="4" max="4" width="12.54296875" style="4" customWidth="1"/>
     <col min="5" max="5" width="15.7265625" style="4" customWidth="1"/>
@@ -3545,7 +3594,7 @@
       <c r="E15" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="F15" s="103" t="s">
+      <c r="F15" s="104" t="s">
         <v>59</v>
       </c>
       <c r="G15" s="32" t="s">
@@ -3580,7 +3629,7 @@
       <c r="E16" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="104"/>
+      <c r="F16" s="105"/>
       <c r="G16" s="53" t="s">
         <v>63</v>
       </c>
@@ -3616,7 +3665,7 @@
       <c r="E17" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="104"/>
+      <c r="F17" s="105"/>
       <c r="G17" s="53" t="s">
         <v>67</v>
       </c>
@@ -3649,7 +3698,7 @@
       <c r="E18" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="104"/>
+      <c r="F18" s="105"/>
       <c r="G18" s="53" t="s">
         <v>60</v>
       </c>
@@ -3682,7 +3731,7 @@
       <c r="E19" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="104"/>
+      <c r="F19" s="105"/>
       <c r="G19" s="53" t="s">
         <v>60</v>
       </c>
@@ -3715,7 +3764,7 @@
       <c r="E20" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="104"/>
+      <c r="F20" s="105"/>
       <c r="G20" s="53" t="s">
         <v>63</v>
       </c>
@@ -3888,7 +3937,7 @@
       <c r="E25" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F25" s="110" t="s">
+      <c r="F25" s="112" t="s">
         <v>90</v>
       </c>
       <c r="G25" s="53" t="s">
@@ -3923,7 +3972,7 @@
       <c r="E26" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F26" s="111"/>
+      <c r="F26" s="113"/>
       <c r="G26" s="53" t="s">
         <v>91</v>
       </c>
@@ -3956,7 +4005,7 @@
       <c r="E27" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="111"/>
+      <c r="F27" s="113"/>
       <c r="G27" s="53" t="s">
         <v>96</v>
       </c>
@@ -3989,7 +4038,7 @@
       <c r="E28" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="111"/>
+      <c r="F28" s="113"/>
       <c r="G28" s="53" t="s">
         <v>96</v>
       </c>
@@ -4022,7 +4071,7 @@
       <c r="E29" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F29" s="111"/>
+      <c r="F29" s="113"/>
       <c r="G29" s="53" t="s">
         <v>96</v>
       </c>
@@ -4055,7 +4104,7 @@
       <c r="E30" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F30" s="103"/>
+      <c r="F30" s="104"/>
       <c r="G30" s="53" t="s">
         <v>96</v>
       </c>
@@ -4123,7 +4172,7 @@
       <c r="E32" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="110" t="s">
+      <c r="F32" s="112" t="s">
         <v>111</v>
       </c>
       <c r="G32" s="57" t="s">
@@ -4158,7 +4207,7 @@
       <c r="E33" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F33" s="111"/>
+      <c r="F33" s="113"/>
       <c r="G33" s="57" t="s">
         <v>112</v>
       </c>
@@ -4191,7 +4240,7 @@
       <c r="E34" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F34" s="103"/>
+      <c r="F34" s="104"/>
       <c r="G34" s="57" t="s">
         <v>112</v>
       </c>
@@ -4224,7 +4273,7 @@
       <c r="E35" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="F35" s="113" t="s">
+      <c r="F35" s="114" t="s">
         <v>120</v>
       </c>
       <c r="G35" s="26" t="s">
@@ -4259,7 +4308,7 @@
       <c r="E36" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F36" s="105"/>
+      <c r="F36" s="109"/>
       <c r="G36" s="13" t="s">
         <v>121</v>
       </c>
@@ -4537,7 +4586,7 @@
       <c r="E44" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="F44" s="114" t="s">
+      <c r="F44" s="115" t="s">
         <v>148</v>
       </c>
       <c r="G44" s="61" t="s">
@@ -4572,7 +4621,7 @@
       <c r="E45" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F45" s="108"/>
+      <c r="F45" s="116"/>
       <c r="G45" s="53" t="s">
         <v>149</v>
       </c>
@@ -4605,7 +4654,7 @@
       <c r="E46" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="F46" s="109"/>
+      <c r="F46" s="117"/>
       <c r="G46" s="65" t="s">
         <v>149</v>
       </c>
@@ -4638,7 +4687,7 @@
       <c r="E47" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="F47" s="111" t="s">
+      <c r="F47" s="113" t="s">
         <v>157</v>
       </c>
       <c r="G47" s="32" t="s">
@@ -4673,7 +4722,7 @@
       <c r="E48" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F48" s="111"/>
+      <c r="F48" s="113"/>
       <c r="G48" s="53" t="s">
         <v>158</v>
       </c>
@@ -4706,7 +4755,7 @@
       <c r="E49" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F49" s="103"/>
+      <c r="F49" s="104"/>
       <c r="G49" s="53" t="s">
         <v>158</v>
       </c>
@@ -5334,7 +5383,7 @@
       <c r="E67" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="F67" s="116" t="s">
+      <c r="F67" s="110" t="s">
         <v>245</v>
       </c>
       <c r="G67" s="32" t="s">
@@ -5369,7 +5418,7 @@
       <c r="E68" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F68" s="117"/>
+      <c r="F68" s="111"/>
       <c r="G68" s="53" t="s">
         <v>251</v>
       </c>
@@ -5402,7 +5451,7 @@
       <c r="E69" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F69" s="117"/>
+      <c r="F69" s="111"/>
       <c r="G69" s="53" t="s">
         <v>251</v>
       </c>
@@ -5435,7 +5484,7 @@
       <c r="E70" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="F70" s="103" t="s">
+      <c r="F70" s="104" t="s">
         <v>261</v>
       </c>
       <c r="G70" s="32" t="s">
@@ -5470,7 +5519,7 @@
       <c r="E71" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="F71" s="104"/>
+      <c r="F71" s="105"/>
       <c r="G71" s="53" t="s">
         <v>262</v>
       </c>
@@ -5503,7 +5552,7 @@
       <c r="E72" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F72" s="104"/>
+      <c r="F72" s="105"/>
       <c r="G72" s="53" t="s">
         <v>262</v>
       </c>
@@ -5536,7 +5585,7 @@
       <c r="E73" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F73" s="104"/>
+      <c r="F73" s="105"/>
       <c r="G73" s="53" t="s">
         <v>262</v>
       </c>
@@ -5569,7 +5618,7 @@
       <c r="E74" s="52" t="s">
         <v>271</v>
       </c>
-      <c r="F74" s="104"/>
+      <c r="F74" s="105"/>
       <c r="G74" s="53" t="s">
         <v>262</v>
       </c>
@@ -5602,7 +5651,7 @@
       <c r="E75" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F75" s="115" t="s">
+      <c r="F75" s="108" t="s">
         <v>273</v>
       </c>
       <c r="G75" s="26" t="s">
@@ -5637,7 +5686,7 @@
       <c r="E76" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F76" s="115"/>
+      <c r="F76" s="108"/>
       <c r="G76" s="26" t="s">
         <v>275</v>
       </c>
@@ -5670,7 +5719,7 @@
       <c r="E77" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="F77" s="105"/>
+      <c r="F77" s="109"/>
       <c r="G77" s="26" t="s">
         <v>275</v>
       </c>
@@ -5837,7 +5886,7 @@
       <c r="E82" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="F82" s="112"/>
+      <c r="F82" s="107"/>
       <c r="G82" s="19" t="s">
         <v>282</v>
       </c>
@@ -5870,7 +5919,7 @@
       <c r="E83" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="F83" s="103" t="s">
+      <c r="F83" s="104" t="s">
         <v>294</v>
       </c>
       <c r="G83" s="32" t="s">
@@ -5905,7 +5954,7 @@
       <c r="E84" s="52" t="s">
         <v>271</v>
       </c>
-      <c r="F84" s="104"/>
+      <c r="F84" s="105"/>
       <c r="G84" s="53" t="s">
         <v>295</v>
       </c>
@@ -5938,7 +5987,7 @@
       <c r="E85" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F85" s="104"/>
+      <c r="F85" s="105"/>
       <c r="G85" s="53" t="s">
         <v>295</v>
       </c>
@@ -5971,7 +6020,7 @@
       <c r="E86" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="F86" s="104"/>
+      <c r="F86" s="105"/>
       <c r="G86" s="53" t="s">
         <v>295</v>
       </c>
@@ -6004,7 +6053,7 @@
       <c r="E87" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F87" s="104"/>
+      <c r="F87" s="105"/>
       <c r="G87" s="53" t="s">
         <v>295</v>
       </c>
@@ -6107,7 +6156,7 @@
       <c r="E90" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F90" s="104" t="s">
+      <c r="F90" s="105" t="s">
         <v>313</v>
       </c>
       <c r="G90" s="53" t="s">
@@ -6142,7 +6191,7 @@
       <c r="E91" s="52" t="s">
         <v>271</v>
       </c>
-      <c r="F91" s="104"/>
+      <c r="F91" s="105"/>
       <c r="G91" s="53" t="s">
         <v>314</v>
       </c>
@@ -6175,7 +6224,7 @@
       <c r="E92" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="F92" s="104"/>
+      <c r="F92" s="105"/>
       <c r="G92" s="53" t="s">
         <v>314</v>
       </c>
@@ -6208,7 +6257,7 @@
       <c r="E93" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F93" s="104"/>
+      <c r="F93" s="105"/>
       <c r="G93" s="53" t="s">
         <v>314</v>
       </c>
@@ -6241,7 +6290,7 @@
       <c r="E94" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F94" s="104"/>
+      <c r="F94" s="105"/>
       <c r="G94" s="53" t="s">
         <v>314</v>
       </c>
@@ -6274,7 +6323,7 @@
       <c r="E95" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="F95" s="103" t="s">
+      <c r="F95" s="104" t="s">
         <v>325</v>
       </c>
       <c r="G95" s="32" t="s">
@@ -6309,7 +6358,7 @@
       <c r="E96" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="F96" s="104"/>
+      <c r="F96" s="105"/>
       <c r="G96" s="53" t="s">
         <v>326</v>
       </c>
@@ -6342,7 +6391,7 @@
       <c r="E97" s="52" t="s">
         <v>271</v>
       </c>
-      <c r="F97" s="104"/>
+      <c r="F97" s="105"/>
       <c r="G97" s="53" t="s">
         <v>331</v>
       </c>
@@ -6375,7 +6424,7 @@
       <c r="E98" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F98" s="104"/>
+      <c r="F98" s="105"/>
       <c r="G98" s="53" t="s">
         <v>326</v>
       </c>
@@ -6408,7 +6457,7 @@
       <c r="E99" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F99" s="104"/>
+      <c r="F99" s="105"/>
       <c r="G99" s="53" t="s">
         <v>326</v>
       </c>
@@ -6441,7 +6490,7 @@
       <c r="E100" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="F100" s="107" t="s">
+      <c r="F100" s="118" t="s">
         <v>339</v>
       </c>
       <c r="G100" s="32" t="s">
@@ -6476,7 +6525,7 @@
       <c r="E101" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F101" s="107"/>
+      <c r="F101" s="118"/>
       <c r="G101" s="58" t="s">
         <v>340</v>
       </c>
@@ -6509,7 +6558,7 @@
       <c r="E102" s="52" t="s">
         <v>344</v>
       </c>
-      <c r="F102" s="104" t="s">
+      <c r="F102" s="105" t="s">
         <v>345</v>
       </c>
       <c r="G102" s="53" t="s">
@@ -6544,7 +6593,7 @@
       <c r="E103" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="F103" s="104"/>
+      <c r="F103" s="105"/>
       <c r="G103" s="53" t="s">
         <v>346</v>
       </c>
@@ -6577,7 +6626,7 @@
       <c r="E104" s="52" t="s">
         <v>271</v>
       </c>
-      <c r="F104" s="104"/>
+      <c r="F104" s="105"/>
       <c r="G104" s="53" t="s">
         <v>346</v>
       </c>
@@ -6610,7 +6659,7 @@
       <c r="E105" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F105" s="104"/>
+      <c r="F105" s="105"/>
       <c r="G105" s="96" t="s">
         <v>346</v>
       </c>
@@ -6643,7 +6692,7 @@
       <c r="E106" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F106" s="104"/>
+      <c r="F106" s="105"/>
       <c r="G106" s="96" t="s">
         <v>346</v>
       </c>
@@ -6676,7 +6725,7 @@
       <c r="E107" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F107" s="104"/>
+      <c r="F107" s="105"/>
       <c r="G107" s="53" t="s">
         <v>340</v>
       </c>
@@ -6709,7 +6758,7 @@
       <c r="E108" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="F108" s="104"/>
+      <c r="F108" s="105"/>
       <c r="G108" s="53" t="s">
         <v>340</v>
       </c>
@@ -6742,7 +6791,7 @@
       <c r="E109" s="34" t="s">
         <v>344</v>
       </c>
-      <c r="F109" s="103" t="s">
+      <c r="F109" s="104" t="s">
         <v>359</v>
       </c>
       <c r="G109" s="32" t="s">
@@ -6777,7 +6826,7 @@
       <c r="E110" s="52" t="s">
         <v>271</v>
       </c>
-      <c r="F110" s="104"/>
+      <c r="F110" s="105"/>
       <c r="G110" s="53" t="s">
         <v>360</v>
       </c>
@@ -6810,7 +6859,7 @@
       <c r="E111" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="F111" s="104"/>
+      <c r="F111" s="105"/>
       <c r="G111" s="53" t="s">
         <v>360</v>
       </c>
@@ -6843,7 +6892,7 @@
       <c r="E112" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F112" s="104"/>
+      <c r="F112" s="105"/>
       <c r="G112" s="53" t="s">
         <v>360</v>
       </c>
@@ -6876,7 +6925,7 @@
       <c r="E113" s="52" t="s">
         <v>235</v>
       </c>
-      <c r="F113" s="104"/>
+      <c r="F113" s="105"/>
       <c r="G113" s="53" t="s">
         <v>360</v>
       </c>
@@ -7239,25 +7288,110 @@
         <v>18</v>
       </c>
     </row>
+    <row r="128" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A128" s="98">
+        <v>3</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="C128" s="103" t="s">
+        <v>417</v>
+      </c>
+      <c r="D128" s="101" t="s">
+        <v>418</v>
+      </c>
+      <c r="E128" s="101" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A129" s="98">
+        <v>3</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="C129" s="103" t="s">
+        <v>424</v>
+      </c>
+      <c r="D129" s="101" t="s">
+        <v>419</v>
+      </c>
+      <c r="E129" s="101" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A130" s="98">
+        <v>3</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="C130" s="103" t="s">
+        <v>426</v>
+      </c>
+      <c r="D130" s="101" t="s">
+        <v>420</v>
+      </c>
+      <c r="E130" s="101" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A131" s="98">
+        <v>3</v>
+      </c>
+      <c r="B131" s="103" t="s">
+        <v>427</v>
+      </c>
+      <c r="C131" s="103" t="s">
+        <v>428</v>
+      </c>
+      <c r="D131" s="101" t="s">
+        <v>421</v>
+      </c>
+      <c r="E131" s="101" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A132" s="98">
+        <v>3</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="C132" s="103" t="s">
+        <v>429</v>
+      </c>
+      <c r="D132" s="101" t="s">
+        <v>422</v>
+      </c>
+      <c r="E132" s="101" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L126" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L127" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="16">
+    <mergeCell ref="F109:F113"/>
+    <mergeCell ref="F102:F108"/>
+    <mergeCell ref="F95:F99"/>
+    <mergeCell ref="F100:F101"/>
+    <mergeCell ref="F83:F87"/>
+    <mergeCell ref="F90:F94"/>
     <mergeCell ref="F15:F20"/>
     <mergeCell ref="F78:F82"/>
     <mergeCell ref="F70:F74"/>
     <mergeCell ref="F75:F77"/>
     <mergeCell ref="F67:F69"/>
-    <mergeCell ref="F83:F87"/>
-    <mergeCell ref="F90:F94"/>
     <mergeCell ref="F25:F30"/>
     <mergeCell ref="F32:F34"/>
     <mergeCell ref="F47:F49"/>
     <mergeCell ref="F35:F36"/>
     <mergeCell ref="F44:F46"/>
-    <mergeCell ref="F109:F113"/>
-    <mergeCell ref="F102:F108"/>
-    <mergeCell ref="F95:F99"/>
-    <mergeCell ref="F100:F101"/>
   </mergeCells>
   <phoneticPr fontId="24" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7274,7 +7408,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="36.1796875" customWidth="1"/>
-    <col min="4" max="4" width="22.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
feat: update estacionesSAMADB.xlsx with new data
</commit_message>
<xml_diff>
--- a/estacionesSAMADB.xlsx
+++ b/estacionesSAMADB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29803"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmonto37\Documents\SAMA\Movimientos Masa\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\scgarzonp\Projects\mantenimientoDash\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B0F1ED3-48A0-419F-9BFB-F51642063E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BC80E8-5193-499A-81D4-41A80F588681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrumentos_actualizado" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="439">
   <si>
     <t>GRUPO</t>
   </si>
@@ -1355,6 +1355,15 @@
   </si>
   <si>
     <t>La Pintada</t>
+  </si>
+  <si>
+    <t>Uramita</t>
+  </si>
+  <si>
+    <t>sn_1052</t>
+  </si>
+  <si>
+    <t>Nivel</t>
   </si>
 </sst>
 </file>
@@ -1364,7 +1373,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1721,7 +1730,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="45">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -2283,6 +2292,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2329,7 +2349,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2616,12 +2636,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2658,13 +2688,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2725,9 +2751,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2765,7 +2791,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2871,7 +2897,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3013,7 +3039,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3021,24 +3047,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ134"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="48.75" customHeight="1"/>
+  <dimension ref="A1:AQ135"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="48.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" style="3" customWidth="1"/>
     <col min="8" max="8" width="14" style="3" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" style="4" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" style="4" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="2"/>
+    <col min="9" max="9" width="9.88671875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="13.109375" style="4" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="1" customFormat="1" ht="112.5" customHeight="1">
+    <row r="1" spans="1:43" s="1" customFormat="1" ht="112.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -3105,7 +3131,7 @@
       <c r="AP1" s="2"/>
       <c r="AQ1" s="2"/>
     </row>
-    <row r="2" spans="1:43" ht="58.5" customHeight="1">
+    <row r="2" spans="1:43" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -3140,7 +3166,7 @@
         <v>-75.964771999999996</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="54.75" customHeight="1">
+    <row r="3" spans="1:43" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <v>1</v>
       </c>
@@ -3175,7 +3201,7 @@
         <v>-75.951490000000007</v>
       </c>
     </row>
-    <row r="4" spans="1:43" ht="68.25" customHeight="1">
+    <row r="4" spans="1:43" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3210,14 +3236,14 @@
         <v>-75.878309999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="78.75" customHeight="1">
+    <row r="5" spans="1:43" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18">
         <v>1</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="111" t="s">
+      <c r="C5" s="97" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="20" t="s">
@@ -3245,7 +3271,7 @@
         <v>-75.879779999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:43" ht="48.75" customHeight="1">
+    <row r="6" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="24">
         <v>1</v>
       </c>
@@ -3280,7 +3306,7 @@
         <v>-76.381780000000006</v>
       </c>
     </row>
-    <row r="7" spans="1:43" ht="48.75" customHeight="1">
+    <row r="7" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>1</v>
       </c>
@@ -3315,7 +3341,7 @@
         <v>-76.381619999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:43" ht="48.75" customHeight="1">
+    <row r="8" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18">
         <v>1</v>
       </c>
@@ -3350,7 +3376,7 @@
         <v>-76.382729999999995</v>
       </c>
     </row>
-    <row r="9" spans="1:43" ht="48.75" customHeight="1">
+    <row r="9" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="30">
         <v>1</v>
       </c>
@@ -3385,7 +3411,7 @@
         <v>-75.995779999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:43" ht="48.75" customHeight="1">
+    <row r="10" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
         <v>1</v>
       </c>
@@ -3420,7 +3446,7 @@
         <v>-75.103290000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:43" ht="48.75" customHeight="1">
+    <row r="11" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15">
         <v>1</v>
       </c>
@@ -3455,7 +3481,7 @@
         <v>-75.110259999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:43" ht="48.75" customHeight="1">
+    <row r="12" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15">
         <v>1</v>
       </c>
@@ -3490,7 +3516,7 @@
         <v>-75.121009999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:43" ht="48.75" customHeight="1">
+    <row r="13" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15">
         <v>1</v>
       </c>
@@ -3525,7 +3551,7 @@
         <v>-75.084419999999994</v>
       </c>
     </row>
-    <row r="14" spans="1:43" ht="48.75" customHeight="1">
+    <row r="14" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="43">
         <v>1</v>
       </c>
@@ -3560,7 +3586,7 @@
         <v>-75.084040000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:43" ht="48.75" customHeight="1">
+    <row r="15" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="43">
         <v>1</v>
       </c>
@@ -3576,7 +3602,7 @@
       <c r="E15" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="96" t="s">
+      <c r="F15" s="99" t="s">
         <v>61</v>
       </c>
       <c r="G15" s="31" t="s">
@@ -3595,7 +3621,7 @@
         <v>-74.990210000000005</v>
       </c>
     </row>
-    <row r="16" spans="1:43" ht="48.75" customHeight="1">
+    <row r="16" spans="1:43" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43">
         <v>1</v>
       </c>
@@ -3611,7 +3637,7 @@
       <c r="E16" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="97"/>
+      <c r="F16" s="100"/>
       <c r="G16" s="52" t="s">
         <v>65</v>
       </c>
@@ -3631,7 +3657,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="48.75" customHeight="1">
+    <row r="17" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="43">
         <v>1</v>
       </c>
@@ -3647,7 +3673,7 @@
       <c r="E17" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="97"/>
+      <c r="F17" s="100"/>
       <c r="G17" s="52" t="s">
         <v>69</v>
       </c>
@@ -3664,7 +3690,7 @@
         <v>-74.991169999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="48.75" customHeight="1">
+    <row r="18" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="43">
         <v>1</v>
       </c>
@@ -3680,7 +3706,7 @@
       <c r="E18" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="97"/>
+      <c r="F18" s="100"/>
       <c r="G18" s="52" t="s">
         <v>62</v>
       </c>
@@ -3697,7 +3723,7 @@
         <v>-74.990269999999995</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="48.75" customHeight="1">
+    <row r="19" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="43">
         <v>1</v>
       </c>
@@ -3713,7 +3739,7 @@
       <c r="E19" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="97"/>
+      <c r="F19" s="100"/>
       <c r="G19" s="52" t="s">
         <v>62</v>
       </c>
@@ -3730,7 +3756,7 @@
         <v>-74.989999999999995</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="48.75" customHeight="1">
+    <row r="20" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="43">
         <v>1</v>
       </c>
@@ -3746,7 +3772,7 @@
       <c r="E20" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F20" s="97"/>
+      <c r="F20" s="100"/>
       <c r="G20" s="52" t="s">
         <v>65</v>
       </c>
@@ -3763,7 +3789,7 @@
         <v>-74.992559999999997</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="48.75" customHeight="1">
+    <row r="21" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="43">
         <v>1</v>
       </c>
@@ -3798,7 +3824,7 @@
         <v>-76.493690000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="48.75" customHeight="1">
+    <row r="22" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="43">
         <v>1</v>
       </c>
@@ -3833,7 +3859,7 @@
         <v>-76.383709999999994</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="48.75" customHeight="1">
+    <row r="23" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="43">
         <v>1</v>
       </c>
@@ -3868,7 +3894,7 @@
         <v>-76.386960000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="48.75" customHeight="1">
+    <row r="24" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="43">
         <v>1</v>
       </c>
@@ -3903,7 +3929,7 @@
         <v>-75.113280000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="48.75" customHeight="1">
+    <row r="25" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43">
         <v>1</v>
       </c>
@@ -3919,7 +3945,7 @@
       <c r="E25" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="104" t="s">
+      <c r="F25" s="108" t="s">
         <v>92</v>
       </c>
       <c r="G25" s="52" t="s">
@@ -3938,7 +3964,7 @@
         <v>-76.133399999999995</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="48.75" customHeight="1">
+    <row r="26" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="43">
         <v>1</v>
       </c>
@@ -3954,7 +3980,7 @@
       <c r="E26" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F26" s="105"/>
+      <c r="F26" s="109"/>
       <c r="G26" s="52" t="s">
         <v>93</v>
       </c>
@@ -3971,7 +3997,7 @@
         <v>-76.148690000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="48.75" customHeight="1">
+    <row r="27" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="43">
         <v>1</v>
       </c>
@@ -3987,7 +4013,7 @@
       <c r="E27" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F27" s="105"/>
+      <c r="F27" s="109"/>
       <c r="G27" s="52" t="s">
         <v>98</v>
       </c>
@@ -4004,7 +4030,7 @@
         <v>-76.058229999999995</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="48.75" customHeight="1">
+    <row r="28" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="43">
         <v>1</v>
       </c>
@@ -4020,7 +4046,7 @@
       <c r="E28" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F28" s="105"/>
+      <c r="F28" s="109"/>
       <c r="G28" s="52" t="s">
         <v>98</v>
       </c>
@@ -4037,7 +4063,7 @@
         <v>-76.110029999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="48.75" customHeight="1">
+    <row r="29" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="43">
         <v>1</v>
       </c>
@@ -4053,7 +4079,7 @@
       <c r="E29" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F29" s="105"/>
+      <c r="F29" s="109"/>
       <c r="G29" s="52" t="s">
         <v>98</v>
       </c>
@@ -4070,7 +4096,7 @@
         <v>-76.128230000000002</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="48.75" customHeight="1">
+    <row r="30" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="43">
         <v>1</v>
       </c>
@@ -4086,7 +4112,7 @@
       <c r="E30" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F30" s="96"/>
+      <c r="F30" s="99"/>
       <c r="G30" s="52" t="s">
         <v>98</v>
       </c>
@@ -4103,7 +4129,7 @@
         <v>-76.133629999999997</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="48.75" customHeight="1">
+    <row r="31" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="43">
         <v>2</v>
       </c>
@@ -4138,7 +4164,7 @@
         <v>-75.990629999999996</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="48.75" customHeight="1">
+    <row r="32" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="43">
         <v>2</v>
       </c>
@@ -4154,7 +4180,7 @@
       <c r="E32" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="104" t="s">
+      <c r="F32" s="108" t="s">
         <v>113</v>
       </c>
       <c r="G32" s="56" t="s">
@@ -4173,7 +4199,7 @@
         <v>-75.253579999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="48.75" customHeight="1">
+    <row r="33" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="43">
         <v>2</v>
       </c>
@@ -4189,7 +4215,7 @@
       <c r="E33" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F33" s="105"/>
+      <c r="F33" s="109"/>
       <c r="G33" s="56" t="s">
         <v>114</v>
       </c>
@@ -4206,7 +4232,7 @@
         <v>-75.283011000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="48.75" customHeight="1">
+    <row r="34" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="43">
         <v>2</v>
       </c>
@@ -4222,7 +4248,7 @@
       <c r="E34" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F34" s="96"/>
+      <c r="F34" s="99"/>
       <c r="G34" s="56" t="s">
         <v>114</v>
       </c>
@@ -4239,7 +4265,7 @@
         <v>-75.348669999999998</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="48.75" customHeight="1">
+    <row r="35" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="15">
         <v>2</v>
       </c>
@@ -4255,7 +4281,7 @@
       <c r="E35" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="F35" s="106" t="s">
+      <c r="F35" s="110" t="s">
         <v>122</v>
       </c>
       <c r="G35" s="25" t="s">
@@ -4274,7 +4300,7 @@
         <v>-76.031049999999993</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="48.75" customHeight="1">
+    <row r="36" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="15">
         <v>2</v>
       </c>
@@ -4290,7 +4316,7 @@
       <c r="E36" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="F36" s="101"/>
+      <c r="F36" s="105"/>
       <c r="G36" s="13" t="s">
         <v>123</v>
       </c>
@@ -4307,7 +4333,7 @@
         <v>-76.006169999999997</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="48.75" customHeight="1">
+    <row r="37" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="15">
         <v>2</v>
       </c>
@@ -4342,7 +4368,7 @@
         <v>-76.049760000000006</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="48.75" customHeight="1">
+    <row r="38" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="15">
         <v>2</v>
       </c>
@@ -4377,7 +4403,7 @@
         <v>-75.6721</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="48.75" customHeight="1">
+    <row r="39" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="15">
         <v>2</v>
       </c>
@@ -4412,7 +4438,7 @@
         <v>-75.676299999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="39.75" customHeight="1">
+    <row r="40" spans="1:11" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="15">
         <v>2</v>
       </c>
@@ -4447,7 +4473,7 @@
         <v>-75.675920000000005</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="65.25" customHeight="1">
+    <row r="41" spans="1:11" ht="65.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15">
         <v>2</v>
       </c>
@@ -4482,7 +4508,7 @@
         <v>-75.546210000000002</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="65.25" customHeight="1">
+    <row r="42" spans="1:11" ht="65.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="15">
         <v>2</v>
       </c>
@@ -4517,7 +4543,7 @@
         <v>-75.553830000000005</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="67.5" customHeight="1">
+    <row r="43" spans="1:11" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="48">
         <v>2</v>
       </c>
@@ -4552,7 +4578,7 @@
         <v>-75.555310000000006</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="60" customHeight="1">
+    <row r="44" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10">
         <v>2</v>
       </c>
@@ -4568,7 +4594,7 @@
       <c r="E44" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="F44" s="107" t="s">
+      <c r="F44" s="111" t="s">
         <v>150</v>
       </c>
       <c r="G44" s="60" t="s">
@@ -4587,7 +4613,7 @@
         <v>-74.783990000000003</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="58.5" customHeight="1">
+    <row r="45" spans="1:11" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="43">
         <v>2</v>
       </c>
@@ -4603,7 +4629,7 @@
       <c r="E45" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F45" s="108"/>
+      <c r="F45" s="112"/>
       <c r="G45" s="52" t="s">
         <v>151</v>
       </c>
@@ -4620,7 +4646,7 @@
         <v>-74.727176</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="63.75" customHeight="1">
+    <row r="46" spans="1:11" ht="63.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="21">
         <v>2</v>
       </c>
@@ -4636,7 +4662,7 @@
       <c r="E46" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="F46" s="109"/>
+      <c r="F46" s="113"/>
       <c r="G46" s="64" t="s">
         <v>151</v>
       </c>
@@ -4653,7 +4679,7 @@
         <v>-74.812200000000004</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="48.75" customHeight="1">
+    <row r="47" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="30">
         <v>2</v>
       </c>
@@ -4669,7 +4695,7 @@
       <c r="E47" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="F47" s="105" t="s">
+      <c r="F47" s="109" t="s">
         <v>159</v>
       </c>
       <c r="G47" s="31" t="s">
@@ -4688,7 +4714,7 @@
         <v>-74.860889999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="48.75" customHeight="1">
+    <row r="48" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="43">
         <v>2</v>
       </c>
@@ -4704,7 +4730,7 @@
       <c r="E48" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F48" s="105"/>
+      <c r="F48" s="109"/>
       <c r="G48" s="52" t="s">
         <v>160</v>
       </c>
@@ -4721,7 +4747,7 @@
         <v>-74.867999999999995</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="48.75" customHeight="1">
+    <row r="49" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="43">
         <v>2</v>
       </c>
@@ -4737,7 +4763,7 @@
       <c r="E49" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F49" s="96"/>
+      <c r="F49" s="99"/>
       <c r="G49" s="52" t="s">
         <v>160</v>
       </c>
@@ -4754,7 +4780,7 @@
         <v>-74.866849999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="74.25" customHeight="1">
+    <row r="50" spans="1:11" ht="74.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="15">
         <v>3</v>
       </c>
@@ -4789,7 +4815,7 @@
         <v>-75.240308999999996</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="72.75" customHeight="1">
+    <row r="51" spans="1:11" ht="72.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="15">
         <v>3</v>
       </c>
@@ -4824,7 +4850,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="78" customHeight="1">
+    <row r="52" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="15">
         <v>3</v>
       </c>
@@ -4859,7 +4885,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="48.75" customHeight="1">
+    <row r="53" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="15">
         <v>3</v>
       </c>
@@ -4894,7 +4920,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="48.75" customHeight="1">
+    <row r="54" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="15">
         <v>3</v>
       </c>
@@ -4929,7 +4955,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="48.75" customHeight="1">
+    <row r="55" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="15">
         <v>3</v>
       </c>
@@ -4964,7 +4990,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="63" customHeight="1">
+    <row r="56" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="15">
         <v>3</v>
       </c>
@@ -4999,7 +5025,7 @@
         <v>-75.572299999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="48.75" customHeight="1">
+    <row r="57" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="15">
         <v>3</v>
       </c>
@@ -5034,7 +5060,7 @@
         <v>-75.804950000000005</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="48.75" customHeight="1">
+    <row r="58" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="15">
         <v>3</v>
       </c>
@@ -5069,7 +5095,7 @@
         <v>-75.591933999999995</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="81" customHeight="1">
+    <row r="59" spans="1:11" ht="81" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="15">
         <v>3</v>
       </c>
@@ -5104,7 +5130,7 @@
         <v>-7538492</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="82.5" customHeight="1">
+    <row r="60" spans="1:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="43">
         <v>3</v>
       </c>
@@ -5139,7 +5165,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="48.75" customHeight="1">
+    <row r="61" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="43">
         <v>3</v>
       </c>
@@ -5174,7 +5200,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="48.75" customHeight="1">
+    <row r="62" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="15">
         <v>3</v>
       </c>
@@ -5209,7 +5235,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="48.75" customHeight="1">
+    <row r="63" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="15">
         <v>3</v>
       </c>
@@ -5244,7 +5270,7 @@
         <v>-74.763050000000007</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="48.75" customHeight="1">
+    <row r="64" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="15">
         <v>3</v>
       </c>
@@ -5279,7 +5305,7 @@
         <v>-74.757955999999993</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="48.75" customHeight="1">
+    <row r="65" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="15">
         <v>3</v>
       </c>
@@ -5314,7 +5340,7 @@
         <v>-75.605699000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="57.75" customHeight="1">
+    <row r="66" spans="1:11" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="43">
         <v>3</v>
       </c>
@@ -5349,7 +5375,7 @@
         <v>-75.977599999999995</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="48.75" customHeight="1">
+    <row r="67" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="43">
         <v>3</v>
       </c>
@@ -5365,7 +5391,7 @@
       <c r="E67" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="F67" s="102" t="s">
+      <c r="F67" s="106" t="s">
         <v>248</v>
       </c>
       <c r="G67" s="31" t="s">
@@ -5384,7 +5410,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="48.75" customHeight="1">
+    <row r="68" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="43">
         <v>3</v>
       </c>
@@ -5400,7 +5426,7 @@
       <c r="E68" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F68" s="103"/>
+      <c r="F68" s="107"/>
       <c r="G68" s="52" t="s">
         <v>254</v>
       </c>
@@ -5417,7 +5443,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="48.75" customHeight="1">
+    <row r="69" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="43">
         <v>3</v>
       </c>
@@ -5433,7 +5459,7 @@
       <c r="E69" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F69" s="103"/>
+      <c r="F69" s="107"/>
       <c r="G69" s="52" t="s">
         <v>254</v>
       </c>
@@ -5450,7 +5476,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="48.75" customHeight="1">
+    <row r="70" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="43">
         <v>3</v>
       </c>
@@ -5466,7 +5492,7 @@
       <c r="E70" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="F70" s="96" t="s">
+      <c r="F70" s="99" t="s">
         <v>264</v>
       </c>
       <c r="G70" s="31" t="s">
@@ -5485,7 +5511,7 @@
         <v>-74.808800000000005</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="48.75" customHeight="1">
+    <row r="71" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="43">
         <v>3</v>
       </c>
@@ -5501,7 +5527,7 @@
       <c r="E71" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="F71" s="97"/>
+      <c r="F71" s="100"/>
       <c r="G71" s="52" t="s">
         <v>265</v>
       </c>
@@ -5518,7 +5544,7 @@
         <v>-74.818200000000004</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="48.75" customHeight="1">
+    <row r="72" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="43">
         <v>3</v>
       </c>
@@ -5534,7 +5560,7 @@
       <c r="E72" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F72" s="97"/>
+      <c r="F72" s="100"/>
       <c r="G72" s="52" t="s">
         <v>265</v>
       </c>
@@ -5551,7 +5577,7 @@
         <v>-74.818292999999997</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="48.75" customHeight="1">
+    <row r="73" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="43">
         <v>3</v>
       </c>
@@ -5567,7 +5593,7 @@
       <c r="E73" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F73" s="97"/>
+      <c r="F73" s="100"/>
       <c r="G73" s="52" t="s">
         <v>265</v>
       </c>
@@ -5584,7 +5610,7 @@
         <v>-74.774966000000006</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="48.75" customHeight="1">
+    <row r="74" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="43">
         <v>3</v>
       </c>
@@ -5600,7 +5626,7 @@
       <c r="E74" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="F74" s="97"/>
+      <c r="F74" s="100"/>
       <c r="G74" s="52" t="s">
         <v>265</v>
       </c>
@@ -5617,7 +5643,7 @@
         <v>-74.772418000000002</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="48.75" customHeight="1">
+    <row r="75" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="15">
         <v>3</v>
       </c>
@@ -5633,7 +5659,7 @@
       <c r="E75" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F75" s="100" t="s">
+      <c r="F75" s="104" t="s">
         <v>276</v>
       </c>
       <c r="G75" s="25" t="s">
@@ -5652,7 +5678,7 @@
         <v>-74.256550000000004</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="48.75" customHeight="1">
+    <row r="76" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="15">
         <v>3</v>
       </c>
@@ -5668,7 +5694,7 @@
       <c r="E76" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="F76" s="100"/>
+      <c r="F76" s="104"/>
       <c r="G76" s="25" t="s">
         <v>278</v>
       </c>
@@ -5685,7 +5711,7 @@
         <v>-74.256550000000004</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="48.75" customHeight="1">
+    <row r="77" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="15">
         <v>3</v>
       </c>
@@ -5701,7 +5727,7 @@
       <c r="E77" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F77" s="101"/>
+      <c r="F77" s="105"/>
       <c r="G77" s="25" t="s">
         <v>278</v>
       </c>
@@ -5718,7 +5744,7 @@
         <v>-74.25658</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="48.75" customHeight="1">
+    <row r="78" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="15">
         <v>4</v>
       </c>
@@ -5734,7 +5760,7 @@
       <c r="E78" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F78" s="98" t="s">
+      <c r="F78" s="102" t="s">
         <v>284</v>
       </c>
       <c r="G78" s="13" t="s">
@@ -5753,7 +5779,7 @@
         <v>-76.572187999999997</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="48.75" customHeight="1">
+    <row r="79" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="15">
         <v>4</v>
       </c>
@@ -5769,7 +5795,7 @@
       <c r="E79" s="15" t="s">
         <v>274</v>
       </c>
-      <c r="F79" s="98"/>
+      <c r="F79" s="102"/>
       <c r="G79" s="13" t="s">
         <v>285</v>
       </c>
@@ -5786,7 +5812,7 @@
         <v>-76.622691000000003</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="48.75" customHeight="1">
+    <row r="80" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="15">
         <v>4</v>
       </c>
@@ -5802,7 +5828,7 @@
       <c r="E80" s="15" t="s">
         <v>289</v>
       </c>
-      <c r="F80" s="98"/>
+      <c r="F80" s="102"/>
       <c r="G80" s="13" t="s">
         <v>285</v>
       </c>
@@ -5819,7 +5845,7 @@
         <v>-76.572187999999997</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="48.75" customHeight="1">
+    <row r="81" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="15">
         <v>4</v>
       </c>
@@ -5835,7 +5861,7 @@
       <c r="E81" s="15" t="s">
         <v>238</v>
       </c>
-      <c r="F81" s="98"/>
+      <c r="F81" s="102"/>
       <c r="G81" s="13" t="s">
         <v>285</v>
       </c>
@@ -5852,7 +5878,7 @@
         <v>-76.561713999999995</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="48.75" customHeight="1">
+    <row r="82" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="15">
         <v>4</v>
       </c>
@@ -5868,7 +5894,7 @@
       <c r="E82" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="F82" s="99"/>
+      <c r="F82" s="103"/>
       <c r="G82" s="19" t="s">
         <v>285</v>
       </c>
@@ -5885,7 +5911,7 @@
         <v>-76.637387000000004</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="48.75" customHeight="1">
+    <row r="83" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="43">
         <v>4</v>
       </c>
@@ -5901,7 +5927,7 @@
       <c r="E83" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F83" s="96" t="s">
+      <c r="F83" s="99" t="s">
         <v>297</v>
       </c>
       <c r="G83" s="31" t="s">
@@ -5920,7 +5946,7 @@
         <v>-76.663884999999993</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="48.75" customHeight="1">
+    <row r="84" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="43">
         <v>4</v>
       </c>
@@ -5936,7 +5962,7 @@
       <c r="E84" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="F84" s="97"/>
+      <c r="F84" s="100"/>
       <c r="G84" s="52" t="s">
         <v>298</v>
       </c>
@@ -5953,7 +5979,7 @@
         <v>-76.808819999999997</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="48.75" customHeight="1">
+    <row r="85" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="43">
         <v>4</v>
       </c>
@@ -5969,7 +5995,7 @@
       <c r="E85" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F85" s="97"/>
+      <c r="F85" s="100"/>
       <c r="G85" s="52" t="s">
         <v>298</v>
       </c>
@@ -5986,7 +6012,7 @@
         <v>-76.655600000000007</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="48.75" customHeight="1">
+    <row r="86" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="43">
         <v>4</v>
       </c>
@@ -6002,7 +6028,7 @@
       <c r="E86" s="51" t="s">
         <v>289</v>
       </c>
-      <c r="F86" s="97"/>
+      <c r="F86" s="100"/>
       <c r="G86" s="52" t="s">
         <v>298</v>
       </c>
@@ -6019,7 +6045,7 @@
         <v>-76.663884999999993</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="48.75" customHeight="1">
+    <row r="87" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="43">
         <v>4</v>
       </c>
@@ -6035,7 +6061,7 @@
       <c r="E87" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F87" s="97"/>
+      <c r="F87" s="100"/>
       <c r="G87" s="52" t="s">
         <v>298</v>
       </c>
@@ -6052,7 +6078,7 @@
         <v>-76.554760000000002</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="48.75" customHeight="1">
+    <row r="88" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="43">
         <v>4</v>
       </c>
@@ -6087,7 +6113,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="48.75" customHeight="1">
+    <row r="89" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="43">
         <v>4</v>
       </c>
@@ -6122,7 +6148,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="48.75" customHeight="1">
+    <row r="90" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="43">
         <v>4</v>
       </c>
@@ -6138,7 +6164,7 @@
       <c r="E90" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F90" s="97" t="s">
+      <c r="F90" s="100" t="s">
         <v>316</v>
       </c>
       <c r="G90" s="52" t="s">
@@ -6157,7 +6183,7 @@
         <v>-76.648269999999997</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="48.75" customHeight="1">
+    <row r="91" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="43">
         <v>4</v>
       </c>
@@ -6173,7 +6199,7 @@
       <c r="E91" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="F91" s="97"/>
+      <c r="F91" s="100"/>
       <c r="G91" s="52" t="s">
         <v>317</v>
       </c>
@@ -6190,7 +6216,7 @@
         <v>-76.670125999999996</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="48.75" customHeight="1">
+    <row r="92" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="43">
         <v>4</v>
       </c>
@@ -6206,7 +6232,7 @@
       <c r="E92" s="51" t="s">
         <v>289</v>
       </c>
-      <c r="F92" s="97"/>
+      <c r="F92" s="100"/>
       <c r="G92" s="52" t="s">
         <v>317</v>
       </c>
@@ -6223,7 +6249,7 @@
         <v>-76.648269999999997</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="48.75" customHeight="1">
+    <row r="93" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="43">
         <v>4</v>
       </c>
@@ -6239,7 +6265,7 @@
       <c r="E93" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F93" s="97"/>
+      <c r="F93" s="100"/>
       <c r="G93" s="52" t="s">
         <v>317</v>
       </c>
@@ -6256,7 +6282,7 @@
         <v>-76.681904000000003</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="48.75" customHeight="1">
+    <row r="94" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="43">
         <v>4</v>
       </c>
@@ -6272,7 +6298,7 @@
       <c r="E94" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F94" s="97"/>
+      <c r="F94" s="100"/>
       <c r="G94" s="52" t="s">
         <v>317</v>
       </c>
@@ -6289,7 +6315,7 @@
         <v>-76.619720000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="48.75" customHeight="1">
+    <row r="95" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="43">
         <v>4</v>
       </c>
@@ -6305,7 +6331,7 @@
       <c r="E95" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F95" s="96" t="s">
+      <c r="F95" s="99" t="s">
         <v>328</v>
       </c>
       <c r="G95" s="31" t="s">
@@ -6324,7 +6350,7 @@
         <v>-76.268739999999994</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="48.75" customHeight="1">
+    <row r="96" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="43">
         <v>4</v>
       </c>
@@ -6340,7 +6366,7 @@
       <c r="E96" s="51" t="s">
         <v>289</v>
       </c>
-      <c r="F96" s="97"/>
+      <c r="F96" s="100"/>
       <c r="G96" s="52" t="s">
         <v>329</v>
       </c>
@@ -6357,7 +6383,7 @@
         <v>-76.268739999999994</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="48.75" customHeight="1">
+    <row r="97" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="43">
         <v>4</v>
       </c>
@@ -6373,7 +6399,7 @@
       <c r="E97" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="F97" s="97"/>
+      <c r="F97" s="100"/>
       <c r="G97" s="52" t="s">
         <v>334</v>
       </c>
@@ -6390,7 +6416,7 @@
         <v>-76.268739999999994</v>
       </c>
     </row>
-    <row r="98" spans="1:11" ht="48.75" customHeight="1">
+    <row r="98" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="43">
         <v>4</v>
       </c>
@@ -6406,7 +6432,7 @@
       <c r="E98" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F98" s="97"/>
+      <c r="F98" s="100"/>
       <c r="G98" s="52" t="s">
         <v>329</v>
       </c>
@@ -6423,7 +6449,7 @@
         <v>-76.27064</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="48.75" customHeight="1">
+    <row r="99" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="43">
         <v>4</v>
       </c>
@@ -6439,7 +6465,7 @@
       <c r="E99" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F99" s="97"/>
+      <c r="F99" s="100"/>
       <c r="G99" s="52" t="s">
         <v>329</v>
       </c>
@@ -6456,7 +6482,7 @@
         <v>-76.264679999999998</v>
       </c>
     </row>
-    <row r="100" spans="1:11" ht="48.75" customHeight="1">
+    <row r="100" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="43">
         <v>4</v>
       </c>
@@ -6472,7 +6498,7 @@
       <c r="E100" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="F100" s="110" t="s">
+      <c r="F100" s="101" t="s">
         <v>342</v>
       </c>
       <c r="G100" s="31" t="s">
@@ -6491,7 +6517,7 @@
         <v>-76.516509999999997</v>
       </c>
     </row>
-    <row r="101" spans="1:11" ht="48.75" customHeight="1">
+    <row r="101" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="43">
         <v>4</v>
       </c>
@@ -6507,7 +6533,7 @@
       <c r="E101" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="F101" s="110"/>
+      <c r="F101" s="101"/>
       <c r="G101" s="57" t="s">
         <v>343</v>
       </c>
@@ -6524,7 +6550,7 @@
         <v>-76.516509999999997</v>
       </c>
     </row>
-    <row r="102" spans="1:11" ht="48.75" customHeight="1">
+    <row r="102" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="43">
         <v>4</v>
       </c>
@@ -6540,7 +6566,7 @@
       <c r="E102" s="51" t="s">
         <v>347</v>
       </c>
-      <c r="F102" s="97" t="s">
+      <c r="F102" s="100" t="s">
         <v>348</v>
       </c>
       <c r="G102" s="52" t="s">
@@ -6559,7 +6585,7 @@
         <v>-76.433395000000004</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="48.75" customHeight="1">
+    <row r="103" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="43">
         <v>4</v>
       </c>
@@ -6575,7 +6601,7 @@
       <c r="E103" s="51" t="s">
         <v>289</v>
       </c>
-      <c r="F103" s="97"/>
+      <c r="F103" s="100"/>
       <c r="G103" s="52" t="s">
         <v>349</v>
       </c>
@@ -6592,7 +6618,7 @@
         <v>-76.433395000000004</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="48.75" customHeight="1">
+    <row r="104" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="43">
         <v>4</v>
       </c>
@@ -6608,7 +6634,7 @@
       <c r="E104" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="F104" s="97"/>
+      <c r="F104" s="100"/>
       <c r="G104" s="52" t="s">
         <v>349</v>
       </c>
@@ -6625,7 +6651,7 @@
         <v>-76.433395000000004</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="48.75" customHeight="1">
+    <row r="105" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="43">
         <v>4</v>
       </c>
@@ -6641,8 +6667,8 @@
       <c r="E105" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F105" s="97"/>
-      <c r="G105" s="112" t="s">
+      <c r="F105" s="100"/>
+      <c r="G105" s="98" t="s">
         <v>349</v>
       </c>
       <c r="H105" s="47">
@@ -6658,7 +6684,7 @@
         <v>-76.435370000000006</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="48.75" customHeight="1">
+    <row r="106" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="43">
         <v>4</v>
       </c>
@@ -6674,8 +6700,8 @@
       <c r="E106" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F106" s="97"/>
-      <c r="G106" s="112" t="s">
+      <c r="F106" s="100"/>
+      <c r="G106" s="98" t="s">
         <v>349</v>
       </c>
       <c r="H106" s="47">
@@ -6691,7 +6717,7 @@
         <v>-76.489293000000004</v>
       </c>
     </row>
-    <row r="107" spans="1:11" ht="48.75" customHeight="1">
+    <row r="107" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="43">
         <v>4</v>
       </c>
@@ -6707,7 +6733,7 @@
       <c r="E107" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F107" s="97"/>
+      <c r="F107" s="100"/>
       <c r="G107" s="52" t="s">
         <v>343</v>
       </c>
@@ -6724,7 +6750,7 @@
         <v>-76.437741000000003</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="48.75" customHeight="1">
+    <row r="108" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="43">
         <v>4</v>
       </c>
@@ -6740,7 +6766,7 @@
       <c r="E108" s="51" t="s">
         <v>289</v>
       </c>
-      <c r="F108" s="97"/>
+      <c r="F108" s="100"/>
       <c r="G108" s="52" t="s">
         <v>343</v>
       </c>
@@ -6757,7 +6783,7 @@
         <v>-76.437741000000003</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="48.75" customHeight="1">
+    <row r="109" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="43">
         <v>4</v>
       </c>
@@ -6773,7 +6799,7 @@
       <c r="E109" s="33" t="s">
         <v>347</v>
       </c>
-      <c r="F109" s="96" t="s">
+      <c r="F109" s="99" t="s">
         <v>362</v>
       </c>
       <c r="G109" s="31" t="s">
@@ -6792,7 +6818,7 @@
         <v>-76.636439999999993</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="48.75" customHeight="1">
+    <row r="110" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="43">
         <v>4</v>
       </c>
@@ -6808,7 +6834,7 @@
       <c r="E110" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="F110" s="97"/>
+      <c r="F110" s="100"/>
       <c r="G110" s="52" t="s">
         <v>363</v>
       </c>
@@ -6825,7 +6851,7 @@
         <v>-76.69417</v>
       </c>
     </row>
-    <row r="111" spans="1:11" ht="48.75" customHeight="1">
+    <row r="111" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="43">
         <v>4</v>
       </c>
@@ -6841,7 +6867,7 @@
       <c r="E111" s="51" t="s">
         <v>289</v>
       </c>
-      <c r="F111" s="97"/>
+      <c r="F111" s="100"/>
       <c r="G111" s="52" t="s">
         <v>363</v>
       </c>
@@ -6858,7 +6884,7 @@
         <v>-76.636439999999993</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="48.75" customHeight="1">
+    <row r="112" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="43">
         <v>4</v>
       </c>
@@ -6874,7 +6900,7 @@
       <c r="E112" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F112" s="97"/>
+      <c r="F112" s="100"/>
       <c r="G112" s="52" t="s">
         <v>363</v>
       </c>
@@ -6891,7 +6917,7 @@
         <v>-76.716989999999996</v>
       </c>
     </row>
-    <row r="113" spans="1:11" ht="48.75" customHeight="1">
+    <row r="113" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="73">
         <v>4</v>
       </c>
@@ -6907,7 +6933,7 @@
       <c r="E113" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F113" s="97"/>
+      <c r="F113" s="100"/>
       <c r="G113" s="52" t="s">
         <v>363</v>
       </c>
@@ -6924,7 +6950,7 @@
         <v>-76.635649999999998</v>
       </c>
     </row>
-    <row r="114" spans="1:11" ht="48.75" customHeight="1">
+    <row r="114" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="51">
         <v>5</v>
       </c>
@@ -6959,7 +6985,7 @@
         <v>-75.452619999999996</v>
       </c>
     </row>
-    <row r="115" spans="1:11" ht="48.75" customHeight="1">
+    <row r="115" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="51">
         <v>5</v>
       </c>
@@ -6994,7 +7020,7 @@
         <v>-75.430487999999997</v>
       </c>
     </row>
-    <row r="116" spans="1:11" ht="48.75" customHeight="1">
+    <row r="116" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="51">
         <v>5</v>
       </c>
@@ -7029,7 +7055,7 @@
         <v>-75.430487999999997</v>
       </c>
     </row>
-    <row r="117" spans="1:11" ht="48.75" customHeight="1">
+    <row r="117" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="53">
         <v>5</v>
       </c>
@@ -7064,7 +7090,7 @@
         <v>-75.748909999999995</v>
       </c>
     </row>
-    <row r="118" spans="1:11" ht="48.75" customHeight="1">
+    <row r="118" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="51">
         <v>5</v>
       </c>
@@ -7099,32 +7125,32 @@
         <v>-75.777010000000004</v>
       </c>
     </row>
-    <row r="119" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A119" s="51">
+    <row r="119" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="53">
         <v>5</v>
       </c>
-      <c r="B119" s="89" t="s">
+      <c r="B119" s="96" t="s">
         <v>380</v>
       </c>
-      <c r="C119" s="52" t="s">
+      <c r="C119" s="57" t="s">
         <v>386</v>
       </c>
-      <c r="D119" s="51" t="s">
+      <c r="D119" s="53" t="s">
         <v>387</v>
       </c>
-      <c r="E119" s="51" t="s">
+      <c r="E119" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="F119" s="52" t="s">
+      <c r="F119" s="57" t="s">
         <v>183</v>
       </c>
-      <c r="G119" s="52" t="s">
+      <c r="G119" s="57" t="s">
         <v>383</v>
       </c>
-      <c r="H119" s="47">
+      <c r="H119" s="74">
         <v>45195</v>
       </c>
-      <c r="I119" s="58">
+      <c r="I119" s="114">
         <v>719</v>
       </c>
       <c r="J119" s="51">
@@ -7134,308 +7160,388 @@
         <v>-75.811940000000007</v>
       </c>
     </row>
-    <row r="120" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A120" s="51">
+    <row r="120" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="15">
         <v>3</v>
       </c>
-      <c r="B120" s="89" t="s">
+      <c r="B120" s="13" t="s">
         <v>388</v>
       </c>
-      <c r="C120" s="3" t="s">
+      <c r="C120" s="13" t="s">
         <v>389</v>
       </c>
-      <c r="D120" s="33" t="s">
+      <c r="D120" s="15" t="s">
         <v>390</v>
       </c>
-      <c r="E120" s="33" t="s">
+      <c r="E120" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J120" s="51"/>
+      <c r="F120" s="13"/>
+      <c r="G120" s="13"/>
+      <c r="H120" s="13"/>
+      <c r="I120" s="15"/>
+      <c r="J120" s="58"/>
       <c r="K120" s="69"/>
     </row>
-    <row r="121" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A121" s="51">
+    <row r="121" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="15">
         <v>3</v>
       </c>
-      <c r="B121" s="89" t="s">
+      <c r="B121" s="13" t="s">
         <v>391</v>
       </c>
-      <c r="C121" s="3" t="s">
+      <c r="C121" s="13" t="s">
         <v>392</v>
       </c>
-      <c r="D121" s="33" t="s">
+      <c r="D121" s="15" t="s">
         <v>393</v>
       </c>
-      <c r="E121" s="33" t="s">
+      <c r="E121" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J121" s="51"/>
+      <c r="F121" s="13"/>
+      <c r="G121" s="13"/>
+      <c r="H121" s="13"/>
+      <c r="I121" s="15"/>
+      <c r="J121" s="58"/>
       <c r="K121" s="69"/>
     </row>
-    <row r="122" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A122" s="51">
+    <row r="122" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="15">
         <v>1</v>
       </c>
-      <c r="B122" s="89" t="s">
+      <c r="B122" s="13" t="s">
         <v>394</v>
       </c>
-      <c r="C122" s="3" t="s">
+      <c r="C122" s="13" t="s">
         <v>395</v>
       </c>
-      <c r="D122" s="33" t="s">
+      <c r="D122" s="15" t="s">
         <v>396</v>
       </c>
-      <c r="E122" s="33" t="s">
+      <c r="E122" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J122" s="51"/>
+      <c r="F122" s="13"/>
+      <c r="G122" s="13"/>
+      <c r="H122" s="13"/>
+      <c r="I122" s="15"/>
+      <c r="J122" s="58"/>
       <c r="K122" s="69"/>
     </row>
-    <row r="123" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A123" s="51">
+    <row r="123" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="15">
         <v>1</v>
       </c>
-      <c r="B123" s="89" t="s">
+      <c r="B123" s="13" t="s">
         <v>397</v>
       </c>
-      <c r="C123" s="3" t="s">
+      <c r="C123" s="13" t="s">
         <v>398</v>
       </c>
-      <c r="D123" s="33" t="s">
+      <c r="D123" s="15" t="s">
         <v>399</v>
       </c>
-      <c r="E123" s="33" t="s">
+      <c r="E123" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J123" s="51"/>
+      <c r="F123" s="13"/>
+      <c r="G123" s="13"/>
+      <c r="H123" s="13"/>
+      <c r="I123" s="15"/>
+      <c r="J123" s="58"/>
       <c r="K123" s="69"/>
     </row>
-    <row r="124" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A124" s="51">
+    <row r="124" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="15">
         <v>1</v>
       </c>
-      <c r="B124" s="89" t="s">
+      <c r="B124" s="13" t="s">
         <v>400</v>
       </c>
-      <c r="C124" s="3" t="s">
+      <c r="C124" s="13" t="s">
         <v>401</v>
       </c>
-      <c r="D124" s="33" t="s">
+      <c r="D124" s="15" t="s">
         <v>402</v>
       </c>
-      <c r="E124" s="33" t="s">
+      <c r="E124" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J124" s="51"/>
+      <c r="F124" s="13"/>
+      <c r="G124" s="13"/>
+      <c r="H124" s="13"/>
+      <c r="I124" s="15"/>
+      <c r="J124" s="58"/>
       <c r="K124" s="69"/>
     </row>
-    <row r="125" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A125" s="51">
+    <row r="125" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="15">
         <v>1</v>
       </c>
-      <c r="B125" s="89" t="s">
+      <c r="B125" s="13" t="s">
         <v>403</v>
       </c>
-      <c r="C125" s="3" t="s">
+      <c r="C125" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="D125" s="33" t="s">
+      <c r="D125" s="15" t="s">
         <v>405</v>
       </c>
-      <c r="E125" s="33" t="s">
+      <c r="E125" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J125" s="51"/>
+      <c r="F125" s="13"/>
+      <c r="G125" s="13"/>
+      <c r="H125" s="13"/>
+      <c r="I125" s="15"/>
+      <c r="J125" s="58"/>
       <c r="K125" s="69"/>
     </row>
-    <row r="126" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A126" s="51">
+    <row r="126" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="15">
         <v>1</v>
       </c>
-      <c r="B126" s="89" t="s">
+      <c r="B126" s="13" t="s">
         <v>406</v>
       </c>
-      <c r="C126" s="3" t="s">
+      <c r="C126" s="13" t="s">
         <v>407</v>
       </c>
-      <c r="D126" s="33" t="s">
+      <c r="D126" s="15" t="s">
         <v>408</v>
       </c>
-      <c r="E126" s="33" t="s">
+      <c r="E126" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J126" s="51"/>
+      <c r="F126" s="13"/>
+      <c r="G126" s="13"/>
+      <c r="H126" s="13"/>
+      <c r="I126" s="15"/>
+      <c r="J126" s="58"/>
       <c r="K126" s="69"/>
     </row>
-    <row r="127" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A127" s="4">
+    <row r="127" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="15">
         <v>3</v>
       </c>
-      <c r="B127" s="3" t="s">
+      <c r="B127" s="13" t="s">
         <v>409</v>
       </c>
-      <c r="C127" s="3" t="s">
+      <c r="C127" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="D127" s="4" t="s">
+      <c r="D127" s="15" t="s">
         <v>411</v>
       </c>
-      <c r="E127" s="33" t="s">
+      <c r="E127" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J127" s="51"/>
+      <c r="F127" s="13"/>
+      <c r="G127" s="13"/>
+      <c r="H127" s="13"/>
+      <c r="I127" s="15"/>
+      <c r="J127" s="58"/>
       <c r="K127" s="69"/>
     </row>
-    <row r="128" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A128" s="51">
+    <row r="128" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="15">
         <v>3</v>
       </c>
-      <c r="B128" s="3" t="s">
+      <c r="B128" s="13" t="s">
         <v>412</v>
       </c>
-      <c r="C128" s="3" t="s">
+      <c r="C128" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="D128" s="33" t="s">
+      <c r="D128" s="15" t="s">
         <v>414</v>
       </c>
-      <c r="E128" s="33" t="s">
+      <c r="E128" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J128" s="51"/>
+      <c r="F128" s="13"/>
+      <c r="G128" s="13"/>
+      <c r="H128" s="13"/>
+      <c r="I128" s="15"/>
+      <c r="J128" s="58"/>
       <c r="K128" s="69"/>
     </row>
-    <row r="129" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A129" s="51">
+    <row r="129" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="15">
         <v>3</v>
       </c>
-      <c r="B129" s="3" t="s">
+      <c r="B129" s="13" t="s">
         <v>415</v>
       </c>
-      <c r="C129" s="3" t="s">
+      <c r="C129" s="13" t="s">
         <v>416</v>
       </c>
-      <c r="D129" s="33" t="s">
+      <c r="D129" s="15" t="s">
         <v>417</v>
       </c>
-      <c r="E129" s="33" t="s">
+      <c r="E129" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J129" s="51"/>
+      <c r="F129" s="13"/>
+      <c r="G129" s="13"/>
+      <c r="H129" s="13"/>
+      <c r="I129" s="15"/>
+      <c r="J129" s="58"/>
       <c r="K129" s="69"/>
     </row>
-    <row r="130" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A130" s="51">
+    <row r="130" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="15">
         <v>3</v>
       </c>
-      <c r="B130" s="3" t="s">
+      <c r="B130" s="13" t="s">
         <v>418</v>
       </c>
-      <c r="C130" s="3" t="s">
+      <c r="C130" s="13" t="s">
         <v>419</v>
       </c>
-      <c r="D130" s="33" t="s">
+      <c r="D130" s="15" t="s">
         <v>420</v>
       </c>
-      <c r="E130" s="33" t="s">
+      <c r="E130" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J130" s="51"/>
+      <c r="F130" s="13"/>
+      <c r="G130" s="13"/>
+      <c r="H130" s="13"/>
+      <c r="I130" s="15"/>
+      <c r="J130" s="58"/>
       <c r="K130" s="69"/>
     </row>
-    <row r="131" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A131" s="51">
+    <row r="131" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="15">
         <v>3</v>
       </c>
-      <c r="B131" s="3" t="s">
+      <c r="B131" s="13" t="s">
         <v>418</v>
       </c>
-      <c r="C131" s="3" t="s">
+      <c r="C131" s="13" t="s">
         <v>421</v>
       </c>
-      <c r="D131" s="33" t="s">
+      <c r="D131" s="15" t="s">
         <v>422</v>
       </c>
-      <c r="E131" s="33" t="s">
+      <c r="E131" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J131" s="51"/>
+      <c r="F131" s="13"/>
+      <c r="G131" s="13"/>
+      <c r="H131" s="13"/>
+      <c r="I131" s="15"/>
+      <c r="J131" s="58"/>
       <c r="K131" s="69"/>
     </row>
-    <row r="132" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A132" s="51">
+    <row r="132" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="15">
         <v>3</v>
       </c>
-      <c r="B132" s="3" t="s">
+      <c r="B132" s="13" t="s">
         <v>423</v>
       </c>
-      <c r="C132" s="3" t="s">
+      <c r="C132" s="13" t="s">
         <v>424</v>
       </c>
-      <c r="D132" s="33" t="s">
+      <c r="D132" s="15" t="s">
         <v>425</v>
       </c>
-      <c r="E132" s="33" t="s">
+      <c r="E132" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J132" s="51"/>
+      <c r="F132" s="13"/>
+      <c r="G132" s="13"/>
+      <c r="H132" s="13"/>
+      <c r="I132" s="15"/>
+      <c r="J132" s="58"/>
       <c r="K132" s="69"/>
     </row>
-    <row r="133" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A133" s="4">
+    <row r="133" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="15">
         <v>3</v>
       </c>
-      <c r="B133" s="3" t="s">
+      <c r="B133" s="13" t="s">
         <v>426</v>
       </c>
-      <c r="C133" s="3" t="s">
+      <c r="C133" s="13" t="s">
         <v>427</v>
       </c>
-      <c r="D133" s="4" t="s">
+      <c r="D133" s="15" t="s">
         <v>428</v>
       </c>
-      <c r="E133" s="33" t="s">
+      <c r="E133" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J133" s="51">
+      <c r="F133" s="13"/>
+      <c r="G133" s="13"/>
+      <c r="H133" s="13"/>
+      <c r="I133" s="15"/>
+      <c r="J133" s="58">
         <v>6.9243490000000003</v>
       </c>
       <c r="K133" s="69">
         <v>-76.174010999999993</v>
       </c>
     </row>
-    <row r="134" spans="1:11" ht="48.75" customHeight="1">
-      <c r="A134" s="4">
+    <row r="134" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="15">
         <v>3</v>
       </c>
-      <c r="B134" s="3" t="s">
+      <c r="B134" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="C134" s="3" t="s">
+      <c r="C134" s="13" t="s">
         <v>429</v>
       </c>
-      <c r="D134" s="4" t="s">
+      <c r="D134" s="15" t="s">
         <v>430</v>
       </c>
-      <c r="E134" s="51" t="s">
+      <c r="E134" s="15" t="s">
         <v>378</v>
       </c>
-      <c r="J134" s="51">
+      <c r="F134" s="13"/>
+      <c r="G134" s="13"/>
+      <c r="H134" s="13"/>
+      <c r="I134" s="15"/>
+      <c r="J134" s="58">
         <v>6.4981549999999997</v>
       </c>
       <c r="K134" s="69">
         <v>-75.113772999999995</v>
       </c>
     </row>
+    <row r="135" spans="1:11" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="15">
+        <v>1</v>
+      </c>
+      <c r="B135" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="C135" s="13" t="s">
+        <v>436</v>
+      </c>
+      <c r="D135" s="17" t="s">
+        <v>437</v>
+      </c>
+      <c r="E135" s="15" t="s">
+        <v>438</v>
+      </c>
+      <c r="F135" s="13"/>
+      <c r="G135" s="13"/>
+      <c r="H135" s="16"/>
+      <c r="I135" s="15"/>
+      <c r="J135" s="58">
+        <v>6.9182969999999999</v>
+      </c>
+      <c r="K135" s="51">
+        <v>-76.173895000000002</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L132" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="F109:F113"/>
-    <mergeCell ref="F102:F108"/>
-    <mergeCell ref="F95:F99"/>
-    <mergeCell ref="F100:F101"/>
-    <mergeCell ref="F83:F87"/>
-    <mergeCell ref="F90:F94"/>
     <mergeCell ref="F15:F20"/>
     <mergeCell ref="F78:F82"/>
     <mergeCell ref="F70:F74"/>
@@ -7446,6 +7552,12 @@
     <mergeCell ref="F47:F49"/>
     <mergeCell ref="F35:F36"/>
     <mergeCell ref="F44:F46"/>
+    <mergeCell ref="F109:F113"/>
+    <mergeCell ref="F102:F108"/>
+    <mergeCell ref="F95:F99"/>
+    <mergeCell ref="F100:F101"/>
+    <mergeCell ref="F83:F87"/>
+    <mergeCell ref="F90:F94"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7459,14 +7571,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{242EFFB5-A78A-42B3-BEEF-7509803C7217}">
   <dimension ref="B4:D11"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="36.140625" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.109375" customWidth="1"/>
+    <col min="4" max="4" width="22.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:4" ht="15" thickBot="1"/>
-    <row r="5" spans="2:4" ht="15" thickBot="1">
+    <row r="4" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="95" t="s">
         <v>390</v>
       </c>
@@ -7478,7 +7590,7 @@
         <v>SANTO DOMINGO - BELLO</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15" thickBot="1">
+    <row r="6" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="95" t="s">
         <v>393</v>
       </c>
@@ -7490,7 +7602,7 @@
         <v>LLANOGRANDE</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15" thickBot="1">
+    <row r="7" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="95" t="s">
         <v>396</v>
       </c>
@@ -7502,7 +7614,7 @@
         <v>VENECIA</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15" thickBot="1">
+    <row r="8" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="95" t="s">
         <v>399</v>
       </c>
@@ -7514,7 +7626,7 @@
         <v>PUERTO BERRÍO</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15" thickBot="1">
+    <row r="9" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="95" t="s">
         <v>402</v>
       </c>
@@ -7526,7 +7638,7 @@
         <v>BRICEÑO</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15" thickBot="1">
+    <row r="10" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="95" t="s">
         <v>405</v>
       </c>
@@ -7538,7 +7650,7 @@
         <v>CIUDAD BOLÍVAR</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15" thickBot="1">
+    <row r="11" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="95" t="s">
         <v>408</v>
       </c>

</xml_diff>